<commit_message>
Note user is Dutch native speaker, update Ahold Delhaize contact note
</commit_message>
<xml_diff>
--- a/Intership/recruitment_contacts.xlsx
+++ b/Intership/recruitment_contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\georg\OneDrive\Documenten\OneDrive\Hero Claude\Intership\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F59B9352-96E4-463C-A64F-5954D14FAA28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8D2ED2-0617-44D8-A18B-480650EE2EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{8C07CF09-9A1D-4DEF-A2BE-72107BDEAE28}"/>
   </bookViews>
@@ -251,9 +251,6 @@
     <t>Search: 'Recruiter Ahold Delhaize Zaandam' on LinkedIn</t>
   </si>
   <si>
-    <t>Note: most internships require Dutch — check language requirements</t>
-  </si>
-  <si>
     <t>FrieslandCampina</t>
   </si>
   <si>
@@ -339,6 +336,9 @@
   </si>
   <si>
     <t>Operations &amp; supply chain consulting</t>
+  </si>
+  <si>
+    <t>Large retail supply chain — no language barrier</t>
   </si>
 </sst>
 </file>
@@ -1053,147 +1053,147 @@
         <v>70</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B17" t="s">
         <v>7</v>
       </c>
       <c r="C17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" t="s">
         <v>73</v>
       </c>
-      <c r="D17" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>74</v>
-      </c>
-      <c r="F17" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
       </c>
       <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" t="s">
         <v>77</v>
       </c>
-      <c r="D18" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>78</v>
-      </c>
-      <c r="F18" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" t="s">
         <v>80</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>81</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
         <v>82</v>
       </c>
-      <c r="D19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>83</v>
-      </c>
-      <c r="F19" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" t="s">
         <v>85</v>
       </c>
-      <c r="B20" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" t="s">
         <v>86</v>
       </c>
-      <c r="D20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>87</v>
-      </c>
-      <c r="F20" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" t="s">
         <v>89</v>
       </c>
-      <c r="B21" t="s">
-        <v>81</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" t="s">
         <v>90</v>
       </c>
-      <c r="D21" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>91</v>
-      </c>
-      <c r="F21" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" t="s">
         <v>93</v>
       </c>
-      <c r="B22" t="s">
-        <v>81</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" t="s">
         <v>94</v>
       </c>
-      <c r="D22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>95</v>
-      </c>
-      <c r="F22" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" t="s">
         <v>97</v>
       </c>
-      <c r="B23" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" t="s">
         <v>98</v>
       </c>
-      <c r="D23" t="s">
-        <v>9</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>99</v>
-      </c>
-      <c r="F23" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild Excel files with all EV companies and specific openings included
</commit_message>
<xml_diff>
--- a/Intership/recruitment_contacts.xlsx
+++ b/Intership/recruitment_contacts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\georg\OneDrive\Documenten\OneDrive\Hero Claude\Intership\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8D2ED2-0617-44D8-A18B-480650EE2EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{76548321-36B3-47B3-800D-AD602BBCBDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{8C07CF09-9A1D-4DEF-A2BE-72107BDEAE28}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{1BB290C1-E4D6-4536-9F59-8059D5268BA7}"/>
   </bookViews>
   <sheets>
     <sheet name="Recruitment Contacts" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="138">
   <si>
     <t>Company</t>
   </si>
@@ -71,7 +71,7 @@
     <t>Search: 'Recruiter Unilever Rotterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Active supply chain internships in Rotterdam — apply directly on career page</t>
+    <t>Active supply chain internships in Rotterdam</t>
   </si>
   <si>
     <t>Heineken</t>
@@ -86,7 +86,7 @@
     <t>Search: 'Talent Acquisition Heineken Amsterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Email recruiter directly — supply chain internships active in Amsterdam</t>
+    <t>Email recruiter directly — supply chain internships active</t>
   </si>
   <si>
     <t>KLM</t>
@@ -101,7 +101,7 @@
     <t>Search: 'KLM Recruiter Young Talent' on LinkedIn</t>
   </si>
   <si>
-    <t>Dedicated internship section on career page — supply chain ops roles available</t>
+    <t>Dedicated internship section on career page</t>
   </si>
   <si>
     <t>Schiphol Group</t>
@@ -137,7 +137,7 @@
     <t>Search: 'HR Rotterdam The Hague Airport' on LinkedIn</t>
   </si>
   <si>
-    <t>Local and smaller — higher chance of success with open application</t>
+    <t>Local and smaller — higher chance with open application</t>
   </si>
   <si>
     <t>Feyenoord</t>
@@ -152,7 +152,7 @@
     <t>Search: 'HR Manager Feyenoord Rotterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Official internship program exists — feyenoord.com/en/our-club/global-football/internships</t>
+    <t>Official internship program exists</t>
   </si>
   <si>
     <t>Ajax</t>
@@ -176,19 +176,19 @@
     <t>Search: 'Talent Acquisition Nike Hilversum' on LinkedIn</t>
   </si>
   <si>
-    <t>European HQ in Hilversum — supply chain &amp; merchandising roles</t>
+    <t>European HQ in Hilversum</t>
   </si>
   <si>
     <t>Adidas</t>
   </si>
   <si>
-    <t>careers.adidas.com</t>
-  </si>
-  <si>
-    <t>Search: 'HR Recruiter Adidas Amsterdam' on LinkedIn</t>
-  </si>
-  <si>
-    <t>Amsterdam European ops hub</t>
+    <t>jobs.adidas-group.com</t>
+  </si>
+  <si>
+    <t>Search: 'Campus Recruiter Adidas Amsterdam' on LinkedIn</t>
+  </si>
+  <si>
+    <t>SPECIFIC OPENING: Intern Buying eCommerce — Sep 2026 EUR 1200/mo Amsterdam hybrid</t>
   </si>
   <si>
     <t>Pon Holdings</t>
@@ -200,7 +200,7 @@
     <t>pon.com/en/carriere</t>
   </si>
   <si>
-    <t>Search: 'Alies Zeck Pon Logistics' on LinkedIn — she is their interim recruiter</t>
+    <t>Search: 'Alies Zeck Pon Logistics' on LinkedIn</t>
   </si>
   <si>
     <t>Large Dutch family company — VW Audi Porsche Bentley importer</t>
@@ -221,13 +221,16 @@
     <t>Tesla</t>
   </si>
   <si>
+    <t>Automotive (EV)</t>
+  </si>
+  <si>
     <t>tesla.com/careers</t>
   </si>
   <si>
     <t>Search: 'Recruiter Tesla Amsterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Fast-growing — logistics and supply chain ops</t>
+    <t>EV leader — great match given personal EV interest</t>
   </si>
   <si>
     <t>DAF Trucks</t>
@@ -242,6 +245,114 @@
     <t>Truck manufacturing in Eindhoven</t>
   </si>
   <si>
+    <t>BMW Group Netherlands</t>
+  </si>
+  <si>
+    <t>werkenbijbmwgroup.nl</t>
+  </si>
+  <si>
+    <t>Search: 'Recruiter BMW Group Netherlands' on LinkedIn</t>
+  </si>
+  <si>
+    <t>Premium automotive</t>
+  </si>
+  <si>
+    <t>Polestar</t>
+  </si>
+  <si>
+    <t>polestar.teamtailor.com</t>
+  </si>
+  <si>
+    <t>Search: 'Recruiter Polestar Netherlands' on LinkedIn</t>
+  </si>
+  <si>
+    <t>SPECIFIC OPENING: Marketing &amp; Events Intern Sep 2026 — Beesd hybrid needs driver's license</t>
+  </si>
+  <si>
+    <t>Fastned</t>
+  </si>
+  <si>
+    <t>fastned.nl/en/careers</t>
+  </si>
+  <si>
+    <t>Search: 'Recruiter Fastned Amsterdam' on LinkedIn</t>
+  </si>
+  <si>
+    <t>EV charging infrastructure — Amsterdam</t>
+  </si>
+  <si>
+    <t>Ebusco</t>
+  </si>
+  <si>
+    <t>ebusco.com/careers</t>
+  </si>
+  <si>
+    <t>Search: 'HR Ebusco Deurne' on LinkedIn</t>
+  </si>
+  <si>
+    <t>Dutch electric bus maker — supply chain roles</t>
+  </si>
+  <si>
+    <t>Jedlix</t>
+  </si>
+  <si>
+    <t>jedlix.com</t>
+  </si>
+  <si>
+    <t>Search: 'Recruiter Jedlix Rotterdam' on LinkedIn</t>
+  </si>
+  <si>
+    <t>Smart EV charging — Rotterdam area very relevant</t>
+  </si>
+  <si>
+    <t>Rivian</t>
+  </si>
+  <si>
+    <t>rivian.com/careers</t>
+  </si>
+  <si>
+    <t>Search: 'Recruiter Rivian Amsterdam' on LinkedIn</t>
+  </si>
+  <si>
+    <t>US EV brand with EU office in Amsterdam</t>
+  </si>
+  <si>
+    <t>BYD Europe</t>
+  </si>
+  <si>
+    <t>bydeurope.com</t>
+  </si>
+  <si>
+    <t>Search: 'Recruiter BYD Europe Amsterdam' on LinkedIn</t>
+  </si>
+  <si>
+    <t>Fastest growing EV brand in Europe</t>
+  </si>
+  <si>
+    <t>Lightyear</t>
+  </si>
+  <si>
+    <t>lightyear.one/careers</t>
+  </si>
+  <si>
+    <t>Search: 'HR Lightyear Helmond' on LinkedIn</t>
+  </si>
+  <si>
+    <t>Dutch solar EV startup</t>
+  </si>
+  <si>
+    <t>ENZA Motors</t>
+  </si>
+  <si>
+    <t>enzamotors.com</t>
+  </si>
+  <si>
+    <t>Search: 'HR ENZA Motors Dordrecht' on LinkedIn</t>
+  </si>
+  <si>
+    <t>Dutch EV startup near Rotterdam</t>
+  </si>
+  <si>
     <t>Ahold Delhaize</t>
   </si>
   <si>
@@ -251,6 +362,9 @@
     <t>Search: 'Recruiter Ahold Delhaize Zaandam' on LinkedIn</t>
   </si>
   <si>
+    <t>Large retail supply chain</t>
+  </si>
+  <si>
     <t>FrieslandCampina</t>
   </si>
   <si>
@@ -336,9 +450,6 @@
   </si>
   <si>
     <t>Operations &amp; supply chain consulting</t>
-  </si>
-  <si>
-    <t>Large retail supply chain — no language barrier</t>
   </si>
 </sst>
 </file>
@@ -394,15 +505,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD180719-D923-4CC8-BF84-E9333CA9D2A2}" name="RecruitmentContacts" displayName="RecruitmentContacts" ref="A1:F23" totalsRowShown="0">
-  <autoFilter ref="A1:F23" xr:uid="{CD180719-D923-4CC8-BF84-E9333CA9D2A2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AA043E5C-EF5F-4A72-B239-3098FFB588BB}" name="RecruitmentContacts" displayName="RecruitmentContacts" ref="A1:F32" totalsRowShown="0">
+  <autoFilter ref="A1:F32" xr:uid="{AA043E5C-EF5F-4A72-B239-3098FFB588BB}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{FE843772-0FD0-4F3E-BA78-6FB6EEFAD198}" name="Company"/>
-    <tableColumn id="2" xr3:uid="{EB706DB1-7DBA-4715-9797-77EAE5C082C6}" name="Industry"/>
-    <tableColumn id="3" xr3:uid="{DFD12105-A14B-4A96-8E11-84040556C805}" name="Career Page"/>
-    <tableColumn id="4" xr3:uid="{EF4F47EA-7837-41EB-A63B-BFC701064A92}" name="Recruitment Email"/>
-    <tableColumn id="5" xr3:uid="{F4041A6E-9918-42FB-8715-215C1BBD966F}" name="LinkedIn Search Tip"/>
-    <tableColumn id="6" xr3:uid="{2FB64C9B-5940-4C0D-B021-1B9E419A99EC}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{53BD358E-D0AE-4E6E-B5C8-E4A3D34C158B}" name="Company"/>
+    <tableColumn id="2" xr3:uid="{BCC97A49-910D-40A7-9EBE-06576939A40A}" name="Industry"/>
+    <tableColumn id="3" xr3:uid="{FE414F78-847A-4152-BAD0-3F0023378BB2}" name="Career Page"/>
+    <tableColumn id="4" xr3:uid="{CDF40C94-E605-4E96-A02D-890920B46220}" name="Recruitment Email"/>
+    <tableColumn id="5" xr3:uid="{C6D0D6D5-FA21-44C8-A06C-CF9857556093}" name="LinkedIn Search Tip"/>
+    <tableColumn id="6" xr3:uid="{06504E43-1C37-4316-8BCD-F16BB9DA0D9C}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -724,16 +835,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09BA9FAB-6EB3-47E5-8C8B-4D4BC41F0BA1}">
-  <dimension ref="A1:F23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B78102E5-4E99-4A65-9AEA-DB39F1B4937E}">
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="62.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="51.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="77.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1001,199 +1112,379 @@
         <v>60</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
         <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" t="s">
         <v>52</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D15" t="s">
         <v>9</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B16" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D16" t="s">
         <v>9</v>
       </c>
       <c r="E16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
         <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D18" t="s">
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
         <v>9</v>
       </c>
       <c r="E19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D20" t="s">
         <v>9</v>
       </c>
       <c r="E20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D21" t="s">
         <v>9</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D22" t="s">
         <v>9</v>
       </c>
       <c r="E22" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D23" t="s">
         <v>9</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F23" t="s">
-        <v>99</v>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>114</v>
+      </c>
+      <c r="D27" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" t="s">
+        <v>118</v>
+      </c>
+      <c r="C28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>120</v>
+      </c>
+      <c r="F28" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" t="s">
+        <v>124</v>
+      </c>
+      <c r="F29" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C30" t="s">
+        <v>127</v>
+      </c>
+      <c r="D30" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" t="s">
+        <v>128</v>
+      </c>
+      <c r="F30" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" t="s">
+        <v>131</v>
+      </c>
+      <c r="D31" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" t="s">
+        <v>132</v>
+      </c>
+      <c r="F31" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>134</v>
+      </c>
+      <c r="B32" t="s">
+        <v>118</v>
+      </c>
+      <c r="C32" t="s">
+        <v>135</v>
+      </c>
+      <c r="D32" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" t="s">
+        <v>136</v>
+      </c>
+      <c r="F32" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add real recruiter emails to recruitment contacts
</commit_message>
<xml_diff>
--- a/Intership/recruitment_contacts.xlsx
+++ b/Intership/recruitment_contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\georg\OneDrive\Documenten\OneDrive\Hero Claude\Intership\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76548321-36B3-47B3-800D-AD602BBCBDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28247FC4-C9AA-4514-ACF1-A4D5B5EB540B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{1BB290C1-E4D6-4536-9F59-8059D5268BA7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="142">
   <si>
     <t>Company</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Search: 'Recruiter Unilever Rotterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Active supply chain internships in Rotterdam</t>
-  </si>
-  <si>
     <t>Heineken</t>
   </si>
   <si>
@@ -86,9 +83,6 @@
     <t>Search: 'Talent Acquisition Heineken Amsterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Email recruiter directly — supply chain internships active</t>
-  </si>
-  <si>
     <t>KLM</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
     <t>Search: 'HR Manager Feyenoord Rotterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>Official internship program exists</t>
-  </si>
-  <si>
     <t>Ajax</t>
   </si>
   <si>
@@ -188,9 +179,6 @@
     <t>Search: 'Campus Recruiter Adidas Amsterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>SPECIFIC OPENING: Intern Buying eCommerce — Sep 2026 EUR 1200/mo Amsterdam hybrid</t>
-  </si>
-  <si>
     <t>Pon Holdings</t>
   </si>
   <si>
@@ -230,9 +218,6 @@
     <t>Search: 'Recruiter Tesla Amsterdam' on LinkedIn</t>
   </si>
   <si>
-    <t>EV leader — great match given personal EV interest</t>
-  </si>
-  <si>
     <t>DAF Trucks</t>
   </si>
   <si>
@@ -450,6 +435,33 @@
   </si>
   <si>
     <t>Operations &amp; supply chain consulting</t>
+  </si>
+  <si>
+    <t>interns.benelux@unilever.com</t>
+  </si>
+  <si>
+    <t>Active supply chain internships in Rotterdam — use internship email directly</t>
+  </si>
+  <si>
+    <t>Direct recruiter email confirmed — supply chain internships active</t>
+  </si>
+  <si>
+    <t>hr@feyenoord.nl (format: first.last@feyenoord.nl)</t>
+  </si>
+  <si>
+    <t>Find recruiter name on LinkedIn then use first.last@feyenoord.nl format</t>
+  </si>
+  <si>
+    <t>Apply via career portal ONLY — no email applications accepted</t>
+  </si>
+  <si>
+    <t>SPECIFIC OPENING: Intern Buying eCommerce Sep 2026 EUR 1200/mo. Deadline Feb/Mar 2026 for Sep start</t>
+  </si>
+  <si>
+    <t>hr@tesla.com</t>
+  </si>
+  <si>
+    <t>EV leader — HR email confirmed. Phone: +31 85 482 2966. Personal EV background is a strong asset</t>
   </si>
 </sst>
 </file>
@@ -842,9 +854,9 @@
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="51.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="77.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="88.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -878,613 +890,613 @@
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>133</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
         <v>23</v>
-      </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E8" t="s">
         <v>35</v>
       </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" t="s">
-        <v>37</v>
-      </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
         <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" t="s">
         <v>43</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>138</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F12" t="s">
         <v>51</v>
-      </c>
-      <c r="B12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
         <v>9</v>
       </c>
       <c r="E13" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F13" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>9</v>
+        <v>140</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F14" t="s">
-        <v>64</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
         <v>9</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
         <v>9</v>
       </c>
       <c r="E16" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
         <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F17" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F18" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
         <v>9</v>
       </c>
       <c r="E19" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F19" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C20" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="D20" t="s">
         <v>9</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F20" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
         <v>9</v>
       </c>
       <c r="E21" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F21" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C22" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D22" t="s">
         <v>9</v>
       </c>
       <c r="E22" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="F22" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C23" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D23" t="s">
         <v>9</v>
       </c>
       <c r="E23" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="F23" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D24" t="s">
         <v>9</v>
       </c>
       <c r="E24" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="F24" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B25" t="s">
         <v>7</v>
       </c>
       <c r="C25" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D25" t="s">
         <v>9</v>
       </c>
       <c r="E25" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="F25" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B26" t="s">
         <v>7</v>
       </c>
       <c r="C26" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D26" t="s">
         <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F26" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B27" t="s">
         <v>7</v>
       </c>
       <c r="C27" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D27" t="s">
         <v>9</v>
       </c>
       <c r="E27" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F27" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C28" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D28" t="s">
         <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F28" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B29" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" t="s">
         <v>118</v>
       </c>
-      <c r="C29" t="s">
-        <v>123</v>
-      </c>
       <c r="D29" t="s">
         <v>9</v>
       </c>
       <c r="E29" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F29" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B30" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
       </c>
       <c r="E30" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="F30" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B31" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D31" t="s">
         <v>9</v>
       </c>
       <c r="E31" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F31" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B32" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C32" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
       </c>
       <c r="E32" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F32" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>